<commit_message>
Correct GBCO: replace study/model/PDF with MNT-Halan-stake-corrected versions (42.58% vs unsourced 20%); update on-site fair value (30.2->37.3, gap -3%->+19%) in data.js/coverage.js, hero + plain-terms + MC-lab copy in EN/AR pages; cache-bust 20260709a
</commit_message>
<xml_diff>
--- a/files/GBCO_Valuation_Model_08072026_public.xlsx
+++ b/files/GBCO_Valuation_Model_08072026_public.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="352">
   <si>
     <t xml:space="preserve">Testahil — GB Corp S.A.E. (EGX: GBCO)</t>
   </si>
@@ -403,7 +403,10 @@
     <t xml:space="preserve">MNT-Halan round valuation (USD mn, Jun-26 first close)</t>
   </si>
   <si>
-    <t xml:space="preserve">GB estimated stake (flagged: not separately published)</t>
+    <t xml:space="preserve">GB stake — last confirmed disclosure (28-Jul-2024 GB Corp PR, fully diluted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORRECTED 09-07-2026: was 0.20 (unsourced estimate, error). GB Corp's own press release states "pre-transactions GBCO's stake in MNT-Halan was 49.45%, ... following the Capital raise ... GBCO's stake shall become 42.58% on a fully diluted basis." Two dilutive events since (a 2024 international raise GB Corp itself participated in pro-rata, and the small Jun-2026 Al Ahly Capital first close, second closing pending) are not individually quantified — flagged as "last confirmed, pre-2026-round," not a guaranteed current figure.</t>
   </si>
   <si>
     <t xml:space="preserve">EGP/USD (study date)</t>
@@ -485,6 +488,30 @@
   </si>
   <si>
     <t xml:space="preserve">The market-implied read: mkt cap − lender − associates ≈ EGP 10.7bn for the Auto leg ≈ 4.0× FY26E Auto EBITDA. Roughly a third of the market value is the MNT-Halan stake, marked to a first-close price.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MNT-Halan stake sensitivity — the crux uncertainty (last confirmed disclosure vs plausible current dilution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GB stake in MNT-Halan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MNT-Halan value (EGP mn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOTP fair value/sh (EGP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prior placeholder (wrong)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">implied by pro-rata defense of the 2024 raise only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last confirmed disclosure (28-Jul-24 PR, pre-2026 dilution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every 5pp of stake ≈ EGP 3.3/share of SOTP fair value — by far the single largest swing factor in this study; confirm the FY25 annual-report associates footnote before relying on any point estimate.</t>
   </si>
   <si>
     <t xml:space="preserve">Segment view — the units × ASP build</t>
@@ -1070,7 +1097,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
@@ -1078,9 +1105,11 @@
     <numFmt numFmtId="168" formatCode="0.00\x"/>
     <numFmt numFmtId="169" formatCode="0.0000%"/>
     <numFmt numFmtId="170" formatCode="@"/>
-    <numFmt numFmtId="171" formatCode="#,##0.0;\(#,##0.0\);\-"/>
-    <numFmt numFmtId="172" formatCode="0.000"/>
-    <numFmt numFmtId="173" formatCode="\+0.0%;\-0.0%;&quot;base&quot;"/>
+    <numFmt numFmtId="171" formatCode="0.0%;\(0.0%\);\-"/>
+    <numFmt numFmtId="172" formatCode="#,##0;\(#,##0\);\-"/>
+    <numFmt numFmtId="173" formatCode="#,##0.0;\(#,##0.0\);\-"/>
+    <numFmt numFmtId="174" formatCode="0.000"/>
+    <numFmt numFmtId="175" formatCode="\+0.0%;\-0.0%;&quot;base&quot;"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -1173,7 +1202,6 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1181,6 +1209,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1246,7 +1275,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1347,7 +1376,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1359,15 +1412,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1387,7 +1440,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1783,7 +1836,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1797,19 +1850,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -1829,7 +1882,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>6937.4</v>
@@ -1863,7 +1916,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>10732.4</v>
@@ -1897,7 +1950,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>7681.4</v>
@@ -1931,7 +1984,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="B9" s="17" t="n">
         <v>6366.1</v>
@@ -1965,7 +2018,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>1743.5</v>
@@ -1999,7 +2052,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="B11" s="17" t="n">
         <v>1039.1</v>
@@ -2033,7 +2086,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>4504.2</v>
@@ -2067,7 +2120,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>3581.4</v>
@@ -2101,17 +2154,17 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="B14" s="30" t="n">
+        <v>253</v>
+      </c>
+      <c r="B14" s="36" t="n">
         <f aca="false">SUM(B6:B13)</f>
         <v>42585.5</v>
       </c>
-      <c r="C14" s="30" t="n">
+      <c r="C14" s="36" t="n">
         <f aca="false">SUM(C6:C13)</f>
         <v>72725.2</v>
       </c>
-      <c r="D14" s="30" t="n">
+      <c r="D14" s="36" t="n">
         <f aca="false">SUM(D6:D13)</f>
         <v>91359</v>
       </c>
@@ -2138,7 +2191,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>19838.8</v>
@@ -2172,7 +2225,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>1363</v>
@@ -2206,7 +2259,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="B18" s="22" t="n">
         <v>21201.8</v>
@@ -2240,7 +2293,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B19" s="17" t="n">
         <v>12517.7</v>
@@ -2274,7 +2327,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>7398.7</v>
@@ -2308,7 +2361,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>371.3</v>
@@ -2342,7 +2395,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="B22" s="17" t="n">
         <v>347.7</v>
@@ -2376,7 +2429,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="B23" s="17" t="n">
         <v>415.2</v>
@@ -2410,7 +2463,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>333.1</v>
@@ -2444,54 +2497,54 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="B25" s="30" t="n">
+        <v>263</v>
+      </c>
+      <c r="B25" s="36" t="n">
         <f aca="false">B18+SUM(B19:B24)</f>
         <v>42585.5</v>
       </c>
-      <c r="C25" s="30" t="n">
+      <c r="C25" s="36" t="n">
         <f aca="false">C18+SUM(C19:C24)</f>
         <v>72725.2</v>
       </c>
-      <c r="D25" s="30" t="n">
+      <c r="D25" s="36" t="n">
         <f aca="false">D18+SUM(D19:D24)</f>
         <v>91359</v>
       </c>
-      <c r="E25" s="30" t="n">
+      <c r="E25" s="36" t="n">
         <f aca="false">E18+SUM(E19:E24)</f>
         <v>103286.500245951</v>
       </c>
-      <c r="F25" s="30" t="n">
+      <c r="F25" s="36" t="n">
         <f aca="false">F18+SUM(F19:F24)</f>
         <v>116573.85008158</v>
       </c>
-      <c r="G25" s="30" t="n">
+      <c r="G25" s="36" t="n">
         <f aca="false">G18+SUM(G19:G24)</f>
         <v>132061.610892388</v>
       </c>
-      <c r="H25" s="30" t="n">
+      <c r="H25" s="36" t="n">
         <f aca="false">H18+SUM(H19:H24)</f>
         <v>149013.658287521</v>
       </c>
-      <c r="I25" s="30" t="n">
+      <c r="I25" s="36" t="n">
         <f aca="false">I18+SUM(I19:I24)</f>
         <v>167485.704726077</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>255</v>
-      </c>
-      <c r="B27" s="31" t="n">
+        <v>264</v>
+      </c>
+      <c r="B27" s="37" t="n">
         <f aca="false">B14-B25</f>
         <v>0</v>
       </c>
-      <c r="C27" s="31" t="n">
+      <c r="C27" s="37" t="n">
         <f aca="false">C14-C25</f>
         <v>0</v>
       </c>
-      <c r="D27" s="31" t="n">
+      <c r="D27" s="37" t="n">
         <f aca="false">D14-D25</f>
         <v>0</v>
       </c>
@@ -2518,7 +2571,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="B28" s="1" t="n">
         <f aca="false">B19-B12</f>
@@ -2555,7 +2608,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B9+B10+B11-(B20-2716.3)</f>
@@ -2592,7 +2645,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="E31" s="8" t="n">
         <f aca="false">E30-D30</f>
@@ -2617,7 +2670,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2645,7 +2698,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2659,7 +2712,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2682,7 +2735,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="E6" s="23" t="n">
         <f aca="false">'Income Statement'!E24</f>
@@ -2707,7 +2760,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="E7" s="23" t="n">
         <f aca="false">'Income Statement'!E18</f>
@@ -2732,7 +2785,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">-'Income Statement'!E16</f>
@@ -2757,7 +2810,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">-'Balance Sheet'!E31</f>
@@ -2782,7 +2835,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="E10" s="23" t="n">
         <f aca="false">-('Balance Sheet'!E8-'Balance Sheet'!D8)</f>
@@ -2807,7 +2860,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="E11" s="22" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -2832,7 +2885,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="E12" s="23" t="n">
         <f aca="false">-Assumptions!$C$57-Assumptions!$C$58</f>
@@ -2857,7 +2910,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="E13" s="22" t="n">
         <f aca="false">E11+E12</f>
@@ -2882,7 +2935,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">Assumptions!$C$71</f>
@@ -2907,7 +2960,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="E15" s="23" t="n">
         <f aca="false">-'Income Statement'!E26*Assumptions!$C$72</f>
@@ -2932,7 +2985,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="E16" s="22" t="n">
         <f aca="false">E13+E14+E15</f>
@@ -2957,7 +3010,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">'Balance Sheet'!D12</f>
@@ -2982,7 +3035,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">E17+E16</f>
@@ -3007,7 +3060,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -3035,7 +3088,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3049,19 +3102,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -3081,7 +3134,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="B6" s="23" t="n">
         <f aca="false">'Income Statement'!B9</f>
@@ -3118,7 +3171,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B7" s="23" t="n">
         <f aca="false">'Income Statement'!B19</f>
@@ -3155,7 +3208,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B8" s="23" t="n">
         <f aca="false">'Income Statement'!B17</f>
@@ -3192,7 +3245,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">'Income Statement'!B26</f>
@@ -3229,7 +3282,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="B10" s="23" t="n">
         <f aca="false">'Balance Sheet'!B14</f>
@@ -3266,7 +3319,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">'Balance Sheet'!B18</f>
@@ -3303,7 +3356,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="B12" s="23" t="n">
         <f aca="false">'Balance Sheet'!B28</f>
@@ -3340,7 +3393,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="E13" s="23" t="n">
         <f aca="false">'Cash Flow'!E13</f>
@@ -3388,7 +3441,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3400,17 +3453,17 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32" t="s">
-        <v>282</v>
+      <c r="A5" s="38" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>0.71394</v>
@@ -3418,109 +3471,109 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>284</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>285</v>
+        <v>293</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>286</v>
-      </c>
-      <c r="B8" s="33" t="s">
-        <v>287</v>
+        <v>295</v>
+      </c>
+      <c r="B8" s="39" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="B9" s="33" t="s">
-        <v>289</v>
+        <v>297</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>291</v>
+        <v>299</v>
+      </c>
+      <c r="B10" s="39" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>299</v>
-      </c>
-      <c r="B14" s="26" t="n">
+        <v>308</v>
+      </c>
+      <c r="B14" s="32" t="n">
         <v>26.1</v>
       </c>
-      <c r="C14" s="26" t="n">
+      <c r="C14" s="32" t="n">
         <v>30</v>
       </c>
-      <c r="D14" s="26" t="n">
+      <c r="D14" s="32" t="n">
         <v>32.5</v>
       </c>
-      <c r="E14" s="26" t="n">
+      <c r="E14" s="32" t="n">
         <v>35.1</v>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="32" t="n">
         <v>40.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="B15" s="26" t="n">
+        <v>309</v>
+      </c>
+      <c r="B15" s="32" t="n">
         <v>24</v>
       </c>
-      <c r="C15" s="26" t="n">
+      <c r="C15" s="32" t="n">
         <v>30.6</v>
       </c>
-      <c r="D15" s="26" t="n">
+      <c r="D15" s="32" t="n">
         <v>35</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="32" t="n">
         <v>40.1</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="32" t="n">
         <v>51.1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">Assumptions!B37</f>
@@ -3529,7 +3582,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B19" s="11" t="n">
         <f aca="false">Assumptions!B38</f>
@@ -3538,7 +3591,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">Assumptions!B39</f>
@@ -3547,22 +3600,22 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="n">
+      <c r="A24" s="32" t="n">
         <v>40</v>
       </c>
       <c r="B24" s="14" t="n">
@@ -3573,7 +3626,7 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="n">
+      <c r="A25" s="32" t="n">
         <v>38</v>
       </c>
       <c r="B25" s="14" t="n">
@@ -3584,7 +3637,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="26" t="n">
+      <c r="A26" s="32" t="n">
         <v>36</v>
       </c>
       <c r="B26" s="14" t="n">
@@ -3595,7 +3648,7 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26" t="n">
+      <c r="A27" s="32" t="n">
         <v>34</v>
       </c>
       <c r="B27" s="14" t="n">
@@ -3606,7 +3659,7 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26" t="n">
+      <c r="A28" s="32" t="n">
         <v>32</v>
       </c>
       <c r="B28" s="14" t="n">
@@ -3617,7 +3670,7 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="26" t="n">
+      <c r="A29" s="32" t="n">
         <v>30</v>
       </c>
       <c r="B29" s="14" t="n">
@@ -3628,7 +3681,7 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="26" t="n">
+      <c r="A30" s="32" t="n">
         <v>28</v>
       </c>
       <c r="B30" s="14" t="n">
@@ -3639,7 +3692,7 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="26" t="n">
+      <c r="A31" s="32" t="n">
         <v>26</v>
       </c>
       <c r="B31" s="14" t="n">
@@ -3674,7 +3727,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3686,157 +3739,157 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="B5" s="34" t="n">
+        <v>320</v>
+      </c>
+      <c r="B5" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C5" s="40" t="n">
         <v>0.05</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="40" t="n">
         <v>0.1</v>
       </c>
-      <c r="E5" s="34" t="n">
+      <c r="E5" s="40" t="n">
         <v>0.15</v>
       </c>
-      <c r="F5" s="34" t="n">
+      <c r="F5" s="40" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="n">
+      <c r="A6" s="41" t="n">
         <v>-0.02</v>
       </c>
-      <c r="B6" s="26" t="n">
+      <c r="B6" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>20.3593200997873</v>
-      </c>
-      <c r="C6" s="26" t="n">
+        <v>34.1927609104736</v>
+      </c>
+      <c r="C6" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>19.3413540947979</v>
-      </c>
-      <c r="D6" s="26" t="n">
+        <v>32.4831228649499</v>
+      </c>
+      <c r="D6" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>18.3233880898086</v>
-      </c>
-      <c r="E6" s="26" t="n">
+        <v>30.7734848194263</v>
+      </c>
+      <c r="E6" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>17.3054220848192</v>
-      </c>
-      <c r="F6" s="26" t="n">
+        <v>29.0638467739026</v>
+      </c>
+      <c r="F6" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>16.2874560798298</v>
+        <v>27.3542087283789</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="n">
+      <c r="A7" s="41" t="n">
         <v>-0.01</v>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>26.1570614182141</v>
-      </c>
-      <c r="C7" s="26" t="n">
+        <v>39.9905022289004</v>
+      </c>
+      <c r="C7" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>24.8492083473034</v>
-      </c>
-      <c r="D7" s="26" t="n">
+        <v>37.9909771174554</v>
+      </c>
+      <c r="D7" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>23.5413552763927</v>
-      </c>
-      <c r="E7" s="26" t="n">
+        <v>35.9914520060104</v>
+      </c>
+      <c r="E7" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>22.233502205482</v>
-      </c>
-      <c r="F7" s="26" t="n">
+        <v>33.9919268945654</v>
+      </c>
+      <c r="F7" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>20.9256491345713</v>
+        <v>31.9924017831204</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="n">
+      <c r="A8" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>31.9548027366409</v>
-      </c>
-      <c r="C8" s="26" t="n">
+        <v>45.7882435473273</v>
+      </c>
+      <c r="C8" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>30.3570625998089</v>
-      </c>
-      <c r="D8" s="26" t="n">
+        <v>43.4988313699609</v>
+      </c>
+      <c r="D8" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>28.7593224629768</v>
-      </c>
-      <c r="E8" s="26" t="n">
+        <v>41.2094191925945</v>
+      </c>
+      <c r="E8" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>27.1615823261448</v>
-      </c>
-      <c r="F8" s="26" t="n">
+        <v>38.9200070152282</v>
+      </c>
+      <c r="F8" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>25.5638421893127</v>
+        <v>36.6305948378618</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="n">
+      <c r="A9" s="41" t="n">
         <v>0.01</v>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>37.7525440550677</v>
-      </c>
-      <c r="C9" s="26" t="n">
+        <v>51.5859848657541</v>
+      </c>
+      <c r="C9" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>35.8649168523144</v>
-      </c>
-      <c r="D9" s="26" t="n">
+        <v>49.0066856224664</v>
+      </c>
+      <c r="D9" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>33.977289649561</v>
-      </c>
-      <c r="E9" s="26" t="n">
+        <v>46.4273863791787</v>
+      </c>
+      <c r="E9" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>32.0896624468076</v>
-      </c>
-      <c r="F9" s="26" t="n">
+        <v>43.848087135891</v>
+      </c>
+      <c r="F9" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>30.2020352440542</v>
+        <v>41.2687878926033</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="n">
+      <c r="A10" s="41" t="n">
         <v>0.02</v>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>43.5502853734946</v>
-      </c>
-      <c r="C10" s="26" t="n">
+        <v>57.3837261841809</v>
+      </c>
+      <c r="C10" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>41.3727711048198</v>
-      </c>
-      <c r="D10" s="26" t="n">
+        <v>54.5145398749718</v>
+      </c>
+      <c r="D10" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>39.1952568361451</v>
-      </c>
-      <c r="E10" s="26" t="n">
+        <v>51.6453535657628</v>
+      </c>
+      <c r="E10" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>37.0177425674704</v>
-      </c>
-      <c r="F10" s="26" t="n">
+        <v>48.7761672565538</v>
+      </c>
+      <c r="F10" s="32" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>34.8402282987957</v>
+        <v>45.9069809473447</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -3864,7 +3917,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3878,19 +3931,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -3910,192 +3963,192 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>315</v>
-      </c>
-      <c r="B6" s="26" t="n">
+        <v>324</v>
+      </c>
+      <c r="B6" s="32" t="n">
         <f aca="false">'Income Statement'!B26/Assumptions!$B$6</f>
         <v>1.74187010594196</v>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="32" t="n">
         <f aca="false">'Income Statement'!C26/Assumptions!$B$6</f>
         <v>2.69746660525104</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="32" t="n">
         <f aca="false">'Income Statement'!D26/Assumptions!$B$6</f>
         <v>2.65315522800553</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="32" t="n">
         <f aca="false">'Income Statement'!E26/Assumptions!$B$6</f>
         <v>3.03778290266124</v>
       </c>
-      <c r="F6" s="26" t="n">
+      <c r="F6" s="32" t="n">
         <f aca="false">'Income Statement'!F26/Assumptions!$B$6</f>
         <v>4.91357065697111</v>
       </c>
-      <c r="G6" s="26" t="n">
+      <c r="G6" s="32" t="n">
         <f aca="false">'Income Statement'!G26/Assumptions!$B$6</f>
         <v>6.88505903961668</v>
       </c>
-      <c r="H6" s="26" t="n">
+      <c r="H6" s="32" t="n">
         <f aca="false">'Income Statement'!H26/Assumptions!$B$6</f>
         <v>8.5758564326992</v>
       </c>
-      <c r="I6" s="26" t="n">
+      <c r="I6" s="32" t="n">
         <f aca="false">'Income Statement'!I26/Assumptions!$B$6</f>
         <v>10.3349758276979</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>316</v>
-      </c>
-      <c r="B7" s="26" t="n">
+        <v>325</v>
+      </c>
+      <c r="B7" s="32" t="n">
         <f aca="false">'Income Statement'!B26*0.13/Assumptions!$B$6</f>
         <v>0.226443113772455</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="32" t="n">
         <f aca="false">'Income Statement'!C26*0.13/Assumptions!$B$6</f>
         <v>0.350670658682635</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="32" t="n">
         <f aca="false">'Income Statement'!D26*0.13/Assumptions!$B$6</f>
         <v>0.344910179640719</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="32" t="n">
         <f aca="false">'Income Statement'!E26*Assumptions!C$72/Assumptions!$B$6</f>
         <v>0.425289606372573</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="32" t="n">
         <f aca="false">'Income Statement'!F26*Assumptions!D$72/Assumptions!$B$6</f>
         <v>0.737035598545666</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="32" t="n">
         <f aca="false">'Income Statement'!G26*Assumptions!E$72/Assumptions!$B$6</f>
         <v>1.10160944633867</v>
       </c>
-      <c r="H7" s="26" t="n">
+      <c r="H7" s="32" t="n">
         <f aca="false">'Income Statement'!H26*Assumptions!F$72/Assumptions!$B$6</f>
         <v>1.54365415788586</v>
       </c>
-      <c r="I7" s="26" t="n">
+      <c r="I7" s="32" t="n">
         <f aca="false">'Income Statement'!I26*Assumptions!G$72/Assumptions!$B$6</f>
         <v>2.06699516553958</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="B8" s="26" t="n">
+        <v>326</v>
+      </c>
+      <c r="B8" s="32" t="n">
         <f aca="false">'Balance Sheet'!B16/Assumptions!$B$6</f>
         <v>18.2761860893597</v>
       </c>
-      <c r="C8" s="26" t="n">
+      <c r="C8" s="32" t="n">
         <f aca="false">'Balance Sheet'!C16/Assumptions!$B$6</f>
         <v>23.4348226623676</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="D8" s="32" t="n">
         <f aca="false">'Balance Sheet'!D16/Assumptions!$B$6</f>
         <v>26.5211423307232</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E8" s="32" t="n">
         <f aca="false">'Balance Sheet'!E16/Assumptions!$B$6</f>
         <v>29.1336356270118</v>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="32" t="n">
         <f aca="false">'Balance Sheet'!F16/Assumptions!$B$6</f>
         <v>33.3101706854373</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="32" t="n">
         <f aca="false">'Balance Sheet'!G16/Assumptions!$B$6</f>
         <v>39.0936202787153</v>
       </c>
-      <c r="H8" s="26" t="n">
+      <c r="H8" s="32" t="n">
         <f aca="false">'Balance Sheet'!H16/Assumptions!$B$6</f>
         <v>46.1258225535286</v>
       </c>
-      <c r="I8" s="26" t="n">
+      <c r="I8" s="32" t="n">
         <f aca="false">'Balance Sheet'!I16/Assumptions!$B$6</f>
         <v>54.3938032156869</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>318</v>
-      </c>
-      <c r="B9" s="27" t="n">
+        <v>327</v>
+      </c>
+      <c r="B9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!B26/Assumptions!$B$6)</f>
         <v>17.9404881531627</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!C26/Assumptions!$B$6)</f>
         <v>11.5849441617431</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!D26/Assumptions!$B$6)</f>
         <v>11.7784288194444</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!E26/Assumptions!$B$6)</f>
         <v>10.2871077365744</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!F26/Assumptions!$B$6)</f>
         <v>6.35993703594436</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!G26/Assumptions!$B$6)</f>
         <v>4.53881365725222</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!H26/Assumptions!$B$6)</f>
         <v>3.643950927262</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!I26/Assumptions!$B$6)</f>
         <v>3.02371292598959</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>319</v>
-      </c>
-      <c r="B10" s="27" t="n">
+        <v>328</v>
+      </c>
+      <c r="B10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!B16/Assumptions!$B$6)</f>
         <v>1.70987534528298</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!C16/Assumptions!$B$6)</f>
         <v>1.33348566149734</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!D16/Assumptions!$B$6)</f>
         <v>1.17830520308315</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!E16/Assumptions!$B$6)</f>
         <v>1.07264333226664</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!F16/Assumptions!$B$6)</f>
         <v>0.938151902465695</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!G16/Assumptions!$B$6)</f>
         <v>0.799363164045828</v>
       </c>
-      <c r="H10" s="27" t="n">
+      <c r="H10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!H16/Assumptions!$B$6)</f>
         <v>0.677494693210829</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!I16/Assumptions!$B$6)</f>
         <v>0.574513973146626</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">B7/Assumptions!$B$5</f>
@@ -4132,7 +4185,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">'Income Statement'!B19/'Income Statement'!B9</f>
@@ -4169,7 +4222,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">'Income Statement'!B26/'Income Statement'!B9</f>
@@ -4206,7 +4259,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">'Income Statement'!B26/'Balance Sheet'!B16</f>
@@ -4243,44 +4296,44 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>324</v>
-      </c>
-      <c r="B15" s="27" t="n">
+        <v>333</v>
+      </c>
+      <c r="B15" s="33" t="n">
         <f aca="false">'Balance Sheet'!B28/'Income Statement'!B19</f>
         <v>1.43367027462206</v>
       </c>
-      <c r="C15" s="27" t="n">
+      <c r="C15" s="33" t="n">
         <f aca="false">'Balance Sheet'!C28/'Income Statement'!C19</f>
         <v>1.96771393405454</v>
       </c>
-      <c r="D15" s="27" t="n">
+      <c r="D15" s="33" t="n">
         <f aca="false">'Balance Sheet'!D28/'Income Statement'!D19</f>
         <v>3.22282369161572</v>
       </c>
-      <c r="E15" s="27" t="n">
+      <c r="E15" s="33" t="n">
         <f aca="false">'Balance Sheet'!E28/'Income Statement'!E19</f>
         <v>3.64511209225965</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="33" t="n">
         <f aca="false">'Balance Sheet'!F28/'Income Statement'!F19</f>
         <v>3.46344101758409</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="33" t="n">
         <f aca="false">'Balance Sheet'!G28/'Income Statement'!G19</f>
         <v>3.21294803033328</v>
       </c>
-      <c r="H15" s="27" t="n">
+      <c r="H15" s="33" t="n">
         <f aca="false">'Balance Sheet'!H28/'Income Statement'!H19</f>
         <v>3.04165844433422</v>
       </c>
-      <c r="I15" s="27" t="n">
+      <c r="I15" s="33" t="n">
         <f aca="false">'Balance Sheet'!I28/'Income Statement'!I19</f>
         <v>2.85450093073083</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14" t="n">
@@ -4314,7 +4367,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14" t="n">
@@ -4348,7 +4401,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
     </row>
   </sheetData>
@@ -4378,7 +4431,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4389,61 +4442,61 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -4505,14 +4558,14 @@
         <v>23</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>13.2</v>
+        <v>22.3</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">SOTP!C14</f>
-        <v>28.7593224629768</v>
+        <v>41.2094191925945</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>50.1</v>
+        <v>66</v>
       </c>
       <c r="E6" s="11" t="n">
         <f aca="false">Assumptions!B32</f>
@@ -4524,14 +4577,14 @@
         <v>24</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>16.1</v>
+        <v>27.2</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">SOTP!C11</f>
-        <v>31.9548027366409</v>
+        <v>45.7882435473273</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>52.2</v>
+        <v>68.8</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">Assumptions!B33</f>
@@ -4582,15 +4635,15 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">SUMPRODUCT(B6:B9,$E$6:$E$9)</f>
-        <v>18.78</v>
+        <v>24.085</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">SUMPRODUCT(C6:C9,$E$6:$E$9)</f>
-        <v>30.2951069267785</v>
+        <v>37.3501617402286</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">SUMPRODUCT(D6:D9,$E$6:$E$9)</f>
-        <v>45.05</v>
+        <v>53.9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4608,7 +4661,7 @@
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">C10/Assumptions!B5-1</f>
-        <v>-0.0305565783430868</v>
+        <v>0.195205175687314</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4675,15 +4728,15 @@
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">Summary!B6</f>
-        <v>13.2</v>
+        <v>22.3</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">Summary!C6</f>
-        <v>28.7593224629768</v>
+        <v>41.2094191925945</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">Summary!D6</f>
-        <v>50.1</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4692,15 +4745,15 @@
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">Summary!B7</f>
-        <v>16.1</v>
+        <v>27.2</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">Summary!C7</f>
-        <v>31.9548027366409</v>
+        <v>45.7882435473273</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">Summary!D7</f>
-        <v>52.2</v>
+        <v>68.8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4743,15 +4796,15 @@
       </c>
       <c r="B10" s="16" t="n">
         <f aca="false">Summary!B10</f>
-        <v>18.78</v>
+        <v>24.085</v>
       </c>
       <c r="C10" s="16" t="n">
         <f aca="false">Summary!C10</f>
-        <v>30.2951069267785</v>
+        <v>37.3501617402286</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">Summary!D10</f>
-        <v>45.05</v>
+        <v>53.9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4970,7 +5023,7 @@
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B79+B80</f>
-        <v>13689.5</v>
+        <v>28705.7</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>61</v>
@@ -5772,12 +5825,15 @@
         <v>122</v>
       </c>
       <c r="B77" s="18" t="n">
-        <v>0.2</v>
+        <v>0.4258</v>
+      </c>
+      <c r="C77" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B78" s="9" t="n">
         <v>47.5</v>
@@ -5785,19 +5841,19 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B79" s="8" t="n">
         <f aca="false">B76*B77*B78</f>
-        <v>13300</v>
+        <v>28315.7</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B80" s="17" t="n">
-        <v>389.5</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -5816,7 +5872,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
@@ -5827,7 +5883,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -5838,26 +5894,26 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C6" s="23" t="n">
         <f aca="false">DCF!B25</f>
@@ -5866,10 +5922,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C7" s="23" t="n">
         <f aca="false">Assumptions!B21*Assumptions!B22</f>
@@ -5878,115 +5934,226 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C8" s="23" t="n">
         <f aca="false">Assumptions!B79*Assumptions!B24</f>
-        <v>13300</v>
+        <v>28315.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C9" s="23" t="n">
         <f aca="false">Assumptions!B80*Assumptions!B24</f>
-        <v>389.5</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="22" t="n">
         <f aca="false">SUM(C6:C9)</f>
-        <v>34686.9383706237</v>
+        <v>49703.1383706237</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="10" t="n">
         <f aca="false">C10/Assumptions!B6</f>
-        <v>31.9548027366409</v>
+        <v>45.7882435473273</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">-C10*Assumptions!B25</f>
-        <v>-3468.69383706237</v>
+        <v>-4970.31383706237</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="22" t="n">
         <f aca="false">C10+C12</f>
-        <v>31218.2445335614</v>
+        <v>44732.8245335614</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="16" t="n">
         <f aca="false">C13/Assumptions!B6</f>
-        <v>28.7593224629768</v>
+        <v>41.2094191925945</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="11" t="n">
         <f aca="false">C14/Assumptions!B5-1</f>
-        <v>-0.0797016811847412</v>
+        <v>0.318701414163025</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">C8/C10</f>
-        <v>0.383429631577509</v>
+        <v>0.569696420150715</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="16" t="n">
         <f aca="false">C8*(1-Assumptions!B25)/Assumptions!B6</f>
-        <v>11.027176416398</v>
+        <v>23.4768585905113</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B22" s="28" t="n">
+        <f aca="false">A22*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>13300</v>
+      </c>
+      <c r="C22" s="29" t="n">
+        <f aca="false">((DCF!$B$25)+B22+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>28.7597370184812</v>
+      </c>
+      <c r="D22" s="30" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B23" s="28" t="n">
+        <f aca="false">A23*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>16625</v>
+      </c>
+      <c r="C23" s="29" t="n">
+        <f aca="false">((DCF!$B$25)+B23+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>31.5165311225807</v>
+      </c>
+      <c r="D23" s="30"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B24" s="28" t="n">
+        <f aca="false">A24*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>19950</v>
+      </c>
+      <c r="C24" s="29" t="n">
+        <f aca="false">((DCF!$B$25)+B24+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>34.2733252266802</v>
+      </c>
+      <c r="D24" s="30"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="27" t="n">
+        <v>0.3545</v>
+      </c>
+      <c r="B25" s="28" t="n">
+        <f aca="false">A25*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>23574.25</v>
+      </c>
+      <c r="C25" s="29" t="n">
+        <f aca="false">((DCF!$B$25)+B25+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>37.2782308001486</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B26" s="28" t="n">
+        <f aca="false">A26*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>26600</v>
+      </c>
+      <c r="C26" s="29" t="n">
+        <f aca="false">((DCF!$B$25)+B26+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>39.7869134348792</v>
+      </c>
+      <c r="D26" s="30"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="n">
+        <v>0.4258</v>
+      </c>
+      <c r="B27" s="28" t="n">
+        <f aca="false">A27*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>28315.7</v>
+      </c>
+      <c r="C27" s="29" t="n">
+        <f aca="false">((DCF!$B$25)+B27+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>41.2094191925945</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -6014,7 +6181,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6028,19 +6195,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -6059,8 +6226,8 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>155</v>
+      <c r="A6" s="31" t="s">
+        <v>164</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>26994</v>
@@ -6093,8 +6260,8 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>155</v>
+      <c r="A7" s="31" t="s">
+        <v>164</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>26994</v>
@@ -6127,8 +6294,8 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>156</v>
+      <c r="A8" s="31" t="s">
+        <v>165</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>16544.3</v>
@@ -6161,45 +6328,45 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>157</v>
-      </c>
-      <c r="B9" s="26" t="n">
+      <c r="A9" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="32" t="n">
         <f aca="false">B8/B7</f>
         <v>0.612888049196118</v>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="32" t="n">
         <f aca="false">C8/C7</f>
         <v>0.86895321456604</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="D9" s="32" t="n">
         <f aca="false">D8/D7</f>
         <v>0.934202801160077</v>
       </c>
-      <c r="E9" s="26" t="n">
+      <c r="E9" s="32" t="n">
         <f aca="false">D9*(1+Assumptions!$C$44)</f>
         <v>0.990254969229681</v>
       </c>
-      <c r="F9" s="26" t="n">
+      <c r="F9" s="32" t="n">
         <f aca="false">E9*(1+Assumptions!$D$44)</f>
         <v>1.05957281707576</v>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="32" t="n">
         <f aca="false">F9*(1+Assumptions!$E$44)</f>
         <v>1.13374291427106</v>
       </c>
-      <c r="H9" s="26" t="n">
+      <c r="H9" s="32" t="n">
         <f aca="false">G9*(1+Assumptions!$F$44)</f>
         <v>1.20176748912733</v>
       </c>
-      <c r="I9" s="26" t="n">
+      <c r="I9" s="32" t="n">
         <f aca="false">H9*(1+Assumptions!$G$44)</f>
         <v>1.27387353847497</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>158</v>
+      <c r="A10" s="31" t="s">
+        <v>167</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>2273</v>
@@ -6232,8 +6399,8 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>159</v>
+      <c r="A11" s="31" t="s">
+        <v>168</v>
       </c>
       <c r="B11" s="17" t="n">
         <v>2323</v>
@@ -6266,8 +6433,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>160</v>
+      <c r="A12" s="31" t="s">
+        <v>169</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>13610</v>
@@ -6300,8 +6467,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>161</v>
+      <c r="A13" s="31" t="s">
+        <v>170</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>854.2</v>
@@ -6334,8 +6501,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>162</v>
+      <c r="A14" s="31" t="s">
+        <v>171</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>2506.8</v>
@@ -6368,8 +6535,8 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>163</v>
+      <c r="A15" s="31" t="s">
+        <v>172</v>
       </c>
       <c r="B15" s="17" t="n">
         <v>7625.2</v>
@@ -6402,8 +6569,8 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
-        <v>164</v>
+      <c r="A16" s="31" t="s">
+        <v>173</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>23854</v>
@@ -6436,8 +6603,8 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>165</v>
+      <c r="A17" s="31" t="s">
+        <v>174</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>4950.9</v>
@@ -6470,8 +6637,8 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>166</v>
+      <c r="A18" s="31" t="s">
+        <v>175</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>-487.7</v>
@@ -6504,8 +6671,8 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
-        <v>167</v>
+      <c r="A19" s="31" t="s">
+        <v>176</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">B16+B17+B18</f>
@@ -6541,8 +6708,8 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
-        <v>168</v>
+      <c r="A21" s="31" t="s">
+        <v>177</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>5813.1</v>
@@ -6575,7 +6742,7 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="31" t="s">
         <v>98</v>
       </c>
       <c r="B22" s="14" t="n">
@@ -6612,8 +6779,8 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>169</v>
+      <c r="A23" s="31" t="s">
+        <v>178</v>
       </c>
       <c r="B23" s="17" t="n">
         <v>3460.9</v>
@@ -6646,8 +6813,8 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25" t="s">
-        <v>170</v>
+      <c r="A24" s="31" t="s">
+        <v>179</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>374.3</v>
@@ -6680,8 +6847,8 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25" t="s">
-        <v>171</v>
+      <c r="A25" s="31" t="s">
+        <v>180</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>3794.6</v>
@@ -6714,8 +6881,8 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
-        <v>172</v>
+      <c r="A26" s="31" t="s">
+        <v>181</v>
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">B25/B16</f>
@@ -6751,8 +6918,8 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="s">
-        <v>173</v>
+      <c r="A27" s="31" t="s">
+        <v>182</v>
       </c>
       <c r="B27" s="17" t="n">
         <v>243.7</v>
@@ -6765,8 +6932,8 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
-        <v>174</v>
+      <c r="A28" s="31" t="s">
+        <v>183</v>
       </c>
       <c r="B28" s="17" t="n">
         <v>1207.6</v>
@@ -6779,8 +6946,8 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25" t="s">
-        <v>175</v>
+      <c r="A29" s="31" t="s">
+        <v>184</v>
       </c>
       <c r="B29" s="17" t="n">
         <v>8980.5</v>
@@ -6794,7 +6961,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -6823,7 +6990,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6834,7 +7001,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6842,18 +7009,18 @@
         <v>33</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">Assumptions!B27*Assumptions!B28/Assumptions!B6</f>
@@ -6862,7 +7029,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">Assumptions!B27/Assumptions!B6</f>
@@ -6871,7 +7038,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">'Income Statement'!E26/Assumptions!B6</f>
@@ -6880,10 +7047,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">Assumptions!B29*Assumptions!B30/Assumptions!B6</f>
@@ -6892,7 +7059,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">Assumptions!B29/Assumptions!B6</f>
@@ -6901,9 +7068,9 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>188</v>
-      </c>
-      <c r="C12" s="27" t="n">
+        <v>197</v>
+      </c>
+      <c r="C12" s="33" t="n">
         <f aca="false">Assumptions!B5/('Balance Sheet'!D16/Assumptions!B6)</f>
         <v>1.17830520308315</v>
       </c>
@@ -6933,7 +7100,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6945,7 +7112,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6967,7 +7134,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B6" s="23" t="n">
         <f aca="false">Segments!E16</f>
@@ -6992,7 +7159,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B7" s="23" t="n">
         <f aca="false">Segments!E25</f>
@@ -7017,7 +7184,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="B8" s="23" t="n">
         <f aca="false">-Segments!E24</f>
@@ -7042,7 +7209,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">Segments!E23</f>
@@ -7067,7 +7234,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B9*(1-Assumptions!$B$7)</f>
@@ -7092,7 +7259,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">Segments!E24</f>
@@ -7117,7 +7284,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">-Assumptions!$C$57</f>
@@ -7142,7 +7309,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B13" s="23" t="n">
         <f aca="false">-'Balance Sheet'!E31</f>
@@ -7167,7 +7334,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">SUM(B10:B13)</f>
@@ -7192,32 +7359,32 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="B15" s="28" t="n">
+        <v>209</v>
+      </c>
+      <c r="B15" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$16)^1</f>
         <v>0.819910711723493</v>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$16)^2</f>
         <v>0.672253575198925</v>
       </c>
-      <c r="D15" s="28" t="n">
+      <c r="D15" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$16)^3</f>
         <v>0.551187907300014</v>
       </c>
-      <c r="E15" s="28" t="n">
+      <c r="E15" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$16)^4</f>
         <v>0.451924869367737</v>
       </c>
-      <c r="F15" s="28" t="n">
+      <c r="F15" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$16)^5</f>
         <v>0.370538041288848</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">B14*B15</f>
@@ -7242,7 +7409,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">SUM(B16:F16)</f>
@@ -7251,7 +7418,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">F14*(1+Assumptions!$B$17)/(Assumptions!$B$16-Assumptions!$B$17)</f>
@@ -7260,7 +7427,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B19*F15</f>
@@ -7269,7 +7436,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">B18+B20</f>
@@ -7278,7 +7445,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="B22" s="24" t="n">
         <f aca="false">B20/B21</f>
@@ -7287,7 +7454,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">-Assumptions!$B$19</f>
@@ -7296,7 +7463,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">-Assumptions!$B$20</f>
@@ -7305,7 +7472,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="B25" s="22" t="n">
         <f aca="false">B21-Assumptions!$B$19-Assumptions!$B$20</f>
@@ -7314,7 +7481,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">0.01*(1-Assumptions!$B$7)*(SUMPRODUCT(B6:F6,B15:F15)+F6*(1+Assumptions!$B$17)/(Assumptions!$B$16-Assumptions!$B$17)*F15)</f>
@@ -7323,7 +7490,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -7351,7 +7518,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7365,19 +7532,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -7397,7 +7564,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>23854</v>
@@ -7431,7 +7598,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>4950.9</v>
@@ -7465,7 +7632,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>-487.7</v>
@@ -7499,15 +7666,15 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="B9" s="29" t="n">
+        <v>224</v>
+      </c>
+      <c r="B9" s="35" t="n">
         <v>28317.2</v>
       </c>
-      <c r="C9" s="29" t="n">
+      <c r="C9" s="35" t="n">
         <v>53969.5</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="35" t="n">
         <v>80229.8</v>
       </c>
       <c r="E9" s="22" t="n">
@@ -7533,7 +7700,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>6884.3</v>
@@ -7567,7 +7734,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">B10/B9</f>
@@ -7604,7 +7771,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>-3430.8</v>
@@ -7638,7 +7805,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>518.8</v>
@@ -7672,7 +7839,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>-268.9</v>
@@ -7706,15 +7873,15 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="B15" s="29" t="n">
+        <v>230</v>
+      </c>
+      <c r="B15" s="35" t="n">
         <v>3703.4</v>
       </c>
-      <c r="C15" s="29" t="n">
+      <c r="C15" s="35" t="n">
         <v>5820.8</v>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="35" t="n">
         <v>6631</v>
       </c>
       <c r="E15" s="22" t="n">
@@ -7740,7 +7907,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>1066.1</v>
@@ -7774,15 +7941,15 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="B17" s="29" t="n">
+        <v>203</v>
+      </c>
+      <c r="B17" s="35" t="n">
         <v>4769.5</v>
       </c>
-      <c r="C17" s="29" t="n">
+      <c r="C17" s="35" t="n">
         <v>6688.5</v>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D17" s="35" t="n">
         <v>7605.7</v>
       </c>
       <c r="E17" s="22" t="n">
@@ -7808,7 +7975,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>820</v>
@@ -7842,7 +8009,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">B17+B18</f>
@@ -7879,7 +8046,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>-1499.2</v>
@@ -7913,7 +8080,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>-965.8</v>
@@ -7947,15 +8114,15 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="B22" s="29" t="n">
+        <v>236</v>
+      </c>
+      <c r="B22" s="35" t="n">
         <v>2304.4</v>
       </c>
-      <c r="C22" s="29" t="n">
+      <c r="C22" s="35" t="n">
         <v>3999.1</v>
       </c>
-      <c r="D22" s="29" t="n">
+      <c r="D22" s="35" t="n">
         <v>3866.5</v>
       </c>
       <c r="E22" s="22" t="n">
@@ -7981,7 +8148,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="B23" s="17" t="n">
         <v>-493.2</v>
@@ -8015,15 +8182,15 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="B24" s="29" t="n">
+        <v>238</v>
+      </c>
+      <c r="B24" s="35" t="n">
         <v>1811.2</v>
       </c>
-      <c r="C24" s="29" t="n">
+      <c r="C24" s="35" t="n">
         <v>3059.9</v>
       </c>
-      <c r="D24" s="29" t="n">
+      <c r="D24" s="35" t="n">
         <v>2780.5</v>
       </c>
       <c r="E24" s="22" t="n">
@@ -8049,7 +8216,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>79.5</v>
@@ -8083,15 +8250,15 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="B26" s="29" t="n">
+        <v>240</v>
+      </c>
+      <c r="B26" s="35" t="n">
         <v>1890.8</v>
       </c>
-      <c r="C26" s="29" t="n">
+      <c r="C26" s="35" t="n">
         <v>2928.1</v>
       </c>
-      <c r="D26" s="29" t="n">
+      <c r="D26" s="35" t="n">
         <v>2880</v>
       </c>
       <c r="E26" s="22" t="n">
@@ -8117,7 +8284,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="B27" s="14" t="n">
         <f aca="false">B26/B9</f>
@@ -8154,7 +8321,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GBCO to confirmed MNT-Halan stake (41.61%, GB Corp PR 9-Jun-2026, superseding the interim 42.58% correction): replace study/model/PDF, update fair value 37.3->37.0 in data.js/coverage.js, hero/plain-terms/MC-lab copy reframed from 'unconfirmed stake' to 'confirmed stake, open discount question'; cache-bust 20260709b
</commit_message>
<xml_diff>
--- a/files/GBCO_Valuation_Model_08072026_public.xlsx
+++ b/files/GBCO_Valuation_Model_08072026_public.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="353">
   <si>
     <t xml:space="preserve">Testahil — GB Corp S.A.E. (EGX: GBCO)</t>
   </si>
@@ -403,10 +403,10 @@
     <t xml:space="preserve">MNT-Halan round valuation (USD mn, Jun-26 first close)</t>
   </si>
   <si>
-    <t xml:space="preserve">GB stake — last confirmed disclosure (28-Jul-2024 GB Corp PR, fully diluted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORRECTED 09-07-2026: was 0.20 (unsourced estimate, error). GB Corp's own press release states "pre-transactions GBCO's stake in MNT-Halan was 49.45%, ... following the Capital raise ... GBCO's stake shall become 42.58% on a fully diluted basis." Two dilutive events since (a 2024 international raise GB Corp itself participated in pro-rata, and the small Jun-2026 Al Ahly Capital first close, second closing pending) are not individually quantified — flagged as "last confirmed, pre-2026-round," not a guaranteed current figure.</t>
+    <t xml:space="preserve">GB stake — CONFIRMED current (GB Corp PR, 9-Jun-2026, post Al Ahly Capital round)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UPDATED 09-07-2026: GB Corp's own press release, 9 June 2026 ("MNT-Halan ... Closes Capital Increase Round Led by Al Ahly Capital Holding"): "GB Corp's ownership stake in MNT-Halan will be adjusted to 41.61%, compared to 42.58% prior to the transaction." This is a current, dated, confirmed figure — not an estimate. Applying it to the round still implies MNT-Halan alone ≈ 82% of GB Corp's market cap; flagged as a genuine valuation puzzle (steep implied private-mark discount, or undervaluation) rather than a sourcing gap.</t>
   </si>
   <si>
     <t xml:space="preserve">EGP/USD (study date)</t>
@@ -490,7 +490,7 @@
     <t xml:space="preserve">The market-implied read: mkt cap − lender − associates ≈ EGP 10.7bn for the Auto leg ≈ 4.0× FY26E Auto EBITDA. Roughly a third of the market value is the MNT-Halan stake, marked to a first-close price.</t>
   </si>
   <si>
-    <t xml:space="preserve">MNT-Halan stake sensitivity — the crux uncertainty (last confirmed disclosure vs plausible current dilution)</t>
+    <t xml:space="preserve">MNT-Halan stake sensitivity — now largely resolved: 41.61% is a confirmed, dated figure (9-Jun-2026)</t>
   </si>
   <si>
     <t xml:space="preserve">GB stake in MNT-Halan</t>
@@ -508,7 +508,10 @@
     <t xml:space="preserve">implied by pro-rata defense of the 2024 raise only</t>
   </si>
   <si>
-    <t xml:space="preserve">last confirmed disclosure (28-Jul-24 PR, pre-2026 dilution)</t>
+    <t xml:space="preserve">superseded — was the pre-transaction figure (28-Jul-2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMED current (GB Corp PR, 9-Jun-2026, post Al Ahly round) — base case</t>
   </si>
   <si>
     <t xml:space="preserve">Every 5pp of stake ≈ EGP 3.3/share of SOTP fair value — by far the single largest swing factor in this study; confirm the FY25 annual-report associates footnote before relying on any point estimate.</t>
@@ -1376,11 +1379,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1401,10 +1408,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1836,7 +1839,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1850,19 +1853,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -1882,7 +1885,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>6937.4</v>
@@ -1916,7 +1919,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>10732.4</v>
@@ -1950,7 +1953,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>7681.4</v>
@@ -1984,7 +1987,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B9" s="17" t="n">
         <v>6366.1</v>
@@ -2018,7 +2021,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>1743.5</v>
@@ -2052,7 +2055,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B11" s="17" t="n">
         <v>1039.1</v>
@@ -2086,7 +2089,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>4504.2</v>
@@ -2120,7 +2123,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>3581.4</v>
@@ -2154,7 +2157,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B14" s="36" t="n">
         <f aca="false">SUM(B6:B13)</f>
@@ -2191,7 +2194,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>19838.8</v>
@@ -2225,7 +2228,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>1363</v>
@@ -2259,7 +2262,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B18" s="22" t="n">
         <v>21201.8</v>
@@ -2293,7 +2296,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B19" s="17" t="n">
         <v>12517.7</v>
@@ -2327,7 +2330,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>7398.7</v>
@@ -2361,7 +2364,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>371.3</v>
@@ -2395,7 +2398,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B22" s="17" t="n">
         <v>347.7</v>
@@ -2429,7 +2432,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B23" s="17" t="n">
         <v>415.2</v>
@@ -2463,7 +2466,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>333.1</v>
@@ -2497,7 +2500,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B25" s="36" t="n">
         <f aca="false">B18+SUM(B19:B24)</f>
@@ -2534,7 +2537,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B27" s="37" t="n">
         <f aca="false">B14-B25</f>
@@ -2571,7 +2574,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B28" s="1" t="n">
         <f aca="false">B19-B12</f>
@@ -2608,7 +2611,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">B9+B10+B11-(B20-2716.3)</f>
@@ -2645,7 +2648,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E31" s="8" t="n">
         <f aca="false">E30-D30</f>
@@ -2670,7 +2673,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -2698,7 +2701,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2712,7 +2715,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2735,7 +2738,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E6" s="23" t="n">
         <f aca="false">'Income Statement'!E24</f>
@@ -2760,7 +2763,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E7" s="23" t="n">
         <f aca="false">'Income Statement'!E18</f>
@@ -2785,7 +2788,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">-'Income Statement'!E16</f>
@@ -2810,7 +2813,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E9" s="23" t="n">
         <f aca="false">-'Balance Sheet'!E31</f>
@@ -2835,7 +2838,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E10" s="23" t="n">
         <f aca="false">-('Balance Sheet'!E8-'Balance Sheet'!D8)</f>
@@ -2860,7 +2863,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E11" s="22" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -2885,7 +2888,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E12" s="23" t="n">
         <f aca="false">-Assumptions!$C$57-Assumptions!$C$58</f>
@@ -2910,7 +2913,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E13" s="22" t="n">
         <f aca="false">E11+E12</f>
@@ -2935,7 +2938,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">Assumptions!$C$71</f>
@@ -2960,7 +2963,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E15" s="23" t="n">
         <f aca="false">-'Income Statement'!E26*Assumptions!$C$72</f>
@@ -2985,7 +2988,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E16" s="22" t="n">
         <f aca="false">E13+E14+E15</f>
@@ -3010,7 +3013,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E17" s="23" t="n">
         <f aca="false">'Balance Sheet'!D12</f>
@@ -3035,7 +3038,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">E17+E16</f>
@@ -3060,7 +3063,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -3088,7 +3091,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3102,19 +3105,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -3134,7 +3137,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B6" s="23" t="n">
         <f aca="false">'Income Statement'!B9</f>
@@ -3171,7 +3174,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B7" s="23" t="n">
         <f aca="false">'Income Statement'!B19</f>
@@ -3208,7 +3211,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B8" s="23" t="n">
         <f aca="false">'Income Statement'!B17</f>
@@ -3245,7 +3248,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">'Income Statement'!B26</f>
@@ -3282,7 +3285,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B10" s="23" t="n">
         <f aca="false">'Balance Sheet'!B14</f>
@@ -3319,7 +3322,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">'Balance Sheet'!B18</f>
@@ -3356,7 +3359,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B12" s="23" t="n">
         <f aca="false">'Balance Sheet'!B28</f>
@@ -3393,7 +3396,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E13" s="23" t="n">
         <f aca="false">'Cash Flow'!E13</f>
@@ -3441,7 +3444,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3453,17 +3456,17 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="38" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>0.71394</v>
@@ -3471,109 +3474,109 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="B14" s="32" t="n">
+        <v>309</v>
+      </c>
+      <c r="B14" s="27" t="n">
         <v>26.1</v>
       </c>
-      <c r="C14" s="32" t="n">
+      <c r="C14" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="D14" s="32" t="n">
+      <c r="D14" s="27" t="n">
         <v>32.5</v>
       </c>
-      <c r="E14" s="32" t="n">
+      <c r="E14" s="27" t="n">
         <v>35.1</v>
       </c>
-      <c r="F14" s="32" t="n">
+      <c r="F14" s="27" t="n">
         <v>40.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="B15" s="32" t="n">
+        <v>310</v>
+      </c>
+      <c r="B15" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="C15" s="32" t="n">
+      <c r="C15" s="27" t="n">
         <v>30.6</v>
       </c>
-      <c r="D15" s="32" t="n">
+      <c r="D15" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="E15" s="32" t="n">
+      <c r="E15" s="27" t="n">
         <v>40.1</v>
       </c>
-      <c r="F15" s="32" t="n">
+      <c r="F15" s="27" t="n">
         <v>51.1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">Assumptions!B37</f>
@@ -3582,7 +3585,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B19" s="11" t="n">
         <f aca="false">Assumptions!B38</f>
@@ -3591,7 +3594,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">Assumptions!B39</f>
@@ -3600,22 +3603,22 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="n">
+      <c r="A24" s="27" t="n">
         <v>40</v>
       </c>
       <c r="B24" s="14" t="n">
@@ -3626,7 +3629,7 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="32" t="n">
+      <c r="A25" s="27" t="n">
         <v>38</v>
       </c>
       <c r="B25" s="14" t="n">
@@ -3637,7 +3640,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="32" t="n">
+      <c r="A26" s="27" t="n">
         <v>36</v>
       </c>
       <c r="B26" s="14" t="n">
@@ -3648,7 +3651,7 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="32" t="n">
+      <c r="A27" s="27" t="n">
         <v>34</v>
       </c>
       <c r="B27" s="14" t="n">
@@ -3659,7 +3662,7 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32" t="n">
+      <c r="A28" s="27" t="n">
         <v>32</v>
       </c>
       <c r="B28" s="14" t="n">
@@ -3670,7 +3673,7 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="32" t="n">
+      <c r="A29" s="27" t="n">
         <v>30</v>
       </c>
       <c r="B29" s="14" t="n">
@@ -3681,7 +3684,7 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32" t="n">
+      <c r="A30" s="27" t="n">
         <v>28</v>
       </c>
       <c r="B30" s="14" t="n">
@@ -3692,7 +3695,7 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="32" t="n">
+      <c r="A31" s="27" t="n">
         <v>26</v>
       </c>
       <c r="B31" s="14" t="n">
@@ -3727,7 +3730,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3739,12 +3742,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B5" s="40" t="n">
         <v>0</v>
@@ -3766,130 +3769,130 @@
       <c r="A6" s="41" t="n">
         <v>-0.02</v>
       </c>
-      <c r="B6" s="32" t="n">
+      <c r="B6" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>34.1927609104736</v>
-      </c>
-      <c r="C6" s="32" t="n">
+        <v>33.5985186258122</v>
+      </c>
+      <c r="C6" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>32.4831228649499</v>
-      </c>
-      <c r="D6" s="32" t="n">
+        <v>31.9185926945216</v>
+      </c>
+      <c r="D6" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>30.7734848194263</v>
-      </c>
-      <c r="E6" s="32" t="n">
+        <v>30.238666763231</v>
+      </c>
+      <c r="E6" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>29.0638467739026</v>
-      </c>
-      <c r="F6" s="32" t="n">
+        <v>28.5587408319403</v>
+      </c>
+      <c r="F6" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A6*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>27.3542087283789</v>
+        <v>26.8788149006497</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="41" t="n">
         <v>-0.01</v>
       </c>
-      <c r="B7" s="32" t="n">
+      <c r="B7" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>39.9905022289004</v>
-      </c>
-      <c r="C7" s="32" t="n">
+        <v>39.396259944239</v>
+      </c>
+      <c r="C7" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>37.9909771174554</v>
-      </c>
-      <c r="D7" s="32" t="n">
+        <v>37.426446947027</v>
+      </c>
+      <c r="D7" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>35.9914520060104</v>
-      </c>
-      <c r="E7" s="32" t="n">
+        <v>35.4566339498151</v>
+      </c>
+      <c r="E7" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>33.9919268945654</v>
-      </c>
-      <c r="F7" s="32" t="n">
+        <v>33.4868209526031</v>
+      </c>
+      <c r="F7" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A7*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>31.9924017831204</v>
+        <v>31.5170079553912</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="B8" s="32" t="n">
+      <c r="B8" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>45.7882435473273</v>
-      </c>
-      <c r="C8" s="32" t="n">
+        <v>45.1940012626658</v>
+      </c>
+      <c r="C8" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>43.4988313699609</v>
-      </c>
-      <c r="D8" s="32" t="n">
+        <v>42.9343011995325</v>
+      </c>
+      <c r="D8" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>41.2094191925945</v>
-      </c>
-      <c r="E8" s="32" t="n">
+        <v>40.6746011363992</v>
+      </c>
+      <c r="E8" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>38.9200070152282</v>
-      </c>
-      <c r="F8" s="32" t="n">
+        <v>38.4149010732659</v>
+      </c>
+      <c r="F8" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A8*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>36.6305948378618</v>
+        <v>36.1552010101327</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="41" t="n">
         <v>0.01</v>
       </c>
-      <c r="B9" s="32" t="n">
+      <c r="B9" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>51.5859848657541</v>
-      </c>
-      <c r="C9" s="32" t="n">
+        <v>50.9917425810926</v>
+      </c>
+      <c r="C9" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>49.0066856224664</v>
-      </c>
-      <c r="D9" s="32" t="n">
+        <v>48.442155452038</v>
+      </c>
+      <c r="D9" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>46.4273863791787</v>
-      </c>
-      <c r="E9" s="32" t="n">
+        <v>45.8925683229834</v>
+      </c>
+      <c r="E9" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>43.848087135891</v>
-      </c>
-      <c r="F9" s="32" t="n">
+        <v>43.3429811939287</v>
+      </c>
+      <c r="F9" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A9*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>41.2687878926033</v>
+        <v>40.7933940648741</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="41" t="n">
         <v>0.02</v>
       </c>
-      <c r="B10" s="32" t="n">
+      <c r="B10" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-B$5))/Assumptions!$B$6</f>
-        <v>57.3837261841809</v>
-      </c>
-      <c r="C10" s="32" t="n">
+        <v>56.7894838995194</v>
+      </c>
+      <c r="C10" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-C$5))/Assumptions!$B$6</f>
-        <v>54.5145398749718</v>
-      </c>
-      <c r="D10" s="32" t="n">
+        <v>53.9500097045435</v>
+      </c>
+      <c r="D10" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-D$5))/Assumptions!$B$6</f>
-        <v>51.6453535657628</v>
-      </c>
-      <c r="E10" s="32" t="n">
+        <v>51.1105355095675</v>
+      </c>
+      <c r="E10" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-E$5))/Assumptions!$B$6</f>
-        <v>48.7761672565538</v>
-      </c>
-      <c r="F10" s="32" t="n">
+        <v>48.2710613145915</v>
+      </c>
+      <c r="F10" s="27" t="n">
         <f aca="false">((DCF!$B$21+$A10*100*DCF!$B$27-Assumptions!$B$19-Assumptions!$B$20+Assumptions!$B$21*Assumptions!$B$22+Assumptions!$B$23*Assumptions!$B$24)*(1-F$5))/Assumptions!$B$6</f>
-        <v>45.9069809473447</v>
+        <v>45.4315871196156</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -3917,7 +3920,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3931,19 +3934,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -3963,118 +3966,118 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>324</v>
-      </c>
-      <c r="B6" s="32" t="n">
+        <v>325</v>
+      </c>
+      <c r="B6" s="27" t="n">
         <f aca="false">'Income Statement'!B26/Assumptions!$B$6</f>
         <v>1.74187010594196</v>
       </c>
-      <c r="C6" s="32" t="n">
+      <c r="C6" s="27" t="n">
         <f aca="false">'Income Statement'!C26/Assumptions!$B$6</f>
         <v>2.69746660525104</v>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="D6" s="27" t="n">
         <f aca="false">'Income Statement'!D26/Assumptions!$B$6</f>
         <v>2.65315522800553</v>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E6" s="27" t="n">
         <f aca="false">'Income Statement'!E26/Assumptions!$B$6</f>
         <v>3.03778290266124</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="27" t="n">
         <f aca="false">'Income Statement'!F26/Assumptions!$B$6</f>
         <v>4.91357065697111</v>
       </c>
-      <c r="G6" s="32" t="n">
+      <c r="G6" s="27" t="n">
         <f aca="false">'Income Statement'!G26/Assumptions!$B$6</f>
         <v>6.88505903961668</v>
       </c>
-      <c r="H6" s="32" t="n">
+      <c r="H6" s="27" t="n">
         <f aca="false">'Income Statement'!H26/Assumptions!$B$6</f>
         <v>8.5758564326992</v>
       </c>
-      <c r="I6" s="32" t="n">
+      <c r="I6" s="27" t="n">
         <f aca="false">'Income Statement'!I26/Assumptions!$B$6</f>
         <v>10.3349758276979</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="B7" s="32" t="n">
+        <v>326</v>
+      </c>
+      <c r="B7" s="27" t="n">
         <f aca="false">'Income Statement'!B26*0.13/Assumptions!$B$6</f>
         <v>0.226443113772455</v>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="27" t="n">
         <f aca="false">'Income Statement'!C26*0.13/Assumptions!$B$6</f>
         <v>0.350670658682635</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="27" t="n">
         <f aca="false">'Income Statement'!D26*0.13/Assumptions!$B$6</f>
         <v>0.344910179640719</v>
       </c>
-      <c r="E7" s="32" t="n">
+      <c r="E7" s="27" t="n">
         <f aca="false">'Income Statement'!E26*Assumptions!C$72/Assumptions!$B$6</f>
         <v>0.425289606372573</v>
       </c>
-      <c r="F7" s="32" t="n">
+      <c r="F7" s="27" t="n">
         <f aca="false">'Income Statement'!F26*Assumptions!D$72/Assumptions!$B$6</f>
         <v>0.737035598545666</v>
       </c>
-      <c r="G7" s="32" t="n">
+      <c r="G7" s="27" t="n">
         <f aca="false">'Income Statement'!G26*Assumptions!E$72/Assumptions!$B$6</f>
         <v>1.10160944633867</v>
       </c>
-      <c r="H7" s="32" t="n">
+      <c r="H7" s="27" t="n">
         <f aca="false">'Income Statement'!H26*Assumptions!F$72/Assumptions!$B$6</f>
         <v>1.54365415788586</v>
       </c>
-      <c r="I7" s="32" t="n">
+      <c r="I7" s="27" t="n">
         <f aca="false">'Income Statement'!I26*Assumptions!G$72/Assumptions!$B$6</f>
         <v>2.06699516553958</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>326</v>
-      </c>
-      <c r="B8" s="32" t="n">
+        <v>327</v>
+      </c>
+      <c r="B8" s="27" t="n">
         <f aca="false">'Balance Sheet'!B16/Assumptions!$B$6</f>
         <v>18.2761860893597</v>
       </c>
-      <c r="C8" s="32" t="n">
+      <c r="C8" s="27" t="n">
         <f aca="false">'Balance Sheet'!C16/Assumptions!$B$6</f>
         <v>23.4348226623676</v>
       </c>
-      <c r="D8" s="32" t="n">
+      <c r="D8" s="27" t="n">
         <f aca="false">'Balance Sheet'!D16/Assumptions!$B$6</f>
         <v>26.5211423307232</v>
       </c>
-      <c r="E8" s="32" t="n">
+      <c r="E8" s="27" t="n">
         <f aca="false">'Balance Sheet'!E16/Assumptions!$B$6</f>
         <v>29.1336356270118</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="27" t="n">
         <f aca="false">'Balance Sheet'!F16/Assumptions!$B$6</f>
         <v>33.3101706854373</v>
       </c>
-      <c r="G8" s="32" t="n">
+      <c r="G8" s="27" t="n">
         <f aca="false">'Balance Sheet'!G16/Assumptions!$B$6</f>
         <v>39.0936202787153</v>
       </c>
-      <c r="H8" s="32" t="n">
+      <c r="H8" s="27" t="n">
         <f aca="false">'Balance Sheet'!H16/Assumptions!$B$6</f>
         <v>46.1258225535286</v>
       </c>
-      <c r="I8" s="32" t="n">
+      <c r="I8" s="27" t="n">
         <f aca="false">'Balance Sheet'!I16/Assumptions!$B$6</f>
         <v>54.3938032156869</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B9" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Income Statement'!B26/Assumptions!$B$6)</f>
@@ -4111,7 +4114,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B10" s="33" t="n">
         <f aca="false">Assumptions!$B$5/('Balance Sheet'!B16/Assumptions!$B$6)</f>
@@ -4148,7 +4151,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">B7/Assumptions!$B$5</f>
@@ -4185,7 +4188,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B12" s="14" t="n">
         <f aca="false">'Income Statement'!B19/'Income Statement'!B9</f>
@@ -4222,7 +4225,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">'Income Statement'!B26/'Income Statement'!B9</f>
@@ -4259,7 +4262,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B14" s="14" t="n">
         <f aca="false">'Income Statement'!B26/'Balance Sheet'!B16</f>
@@ -4296,7 +4299,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B15" s="33" t="n">
         <f aca="false">'Balance Sheet'!B28/'Income Statement'!B19</f>
@@ -4333,7 +4336,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14" t="n">
@@ -4367,7 +4370,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14" t="n">
@@ -4401,7 +4404,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -4431,7 +4434,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4442,7 +4445,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4450,53 +4453,53 @@
         <v>129</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -4558,14 +4561,14 @@
         <v>23</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>22.3</v>
+        <v>21.9</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">SOTP!C14</f>
-        <v>41.2094191925945</v>
+        <v>40.6746011363992</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>66</v>
+        <v>65.4</v>
       </c>
       <c r="E6" s="11" t="n">
         <f aca="false">Assumptions!B32</f>
@@ -4577,14 +4580,14 @@
         <v>24</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">SOTP!C11</f>
-        <v>45.7882435473273</v>
+        <v>45.1940012626658</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>68.8</v>
+        <v>68.1</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">Assumptions!B33</f>
@@ -4635,15 +4638,15 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">SUMPRODUCT(B6:B9,$E$6:$E$9)</f>
-        <v>24.085</v>
+        <v>23.85</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">SUMPRODUCT(C6:C9,$E$6:$E$9)</f>
-        <v>37.3501617402286</v>
+        <v>37.0470981750512</v>
       </c>
       <c r="D10" s="13" t="n">
         <f aca="false">SUMPRODUCT(D6:D9,$E$6:$E$9)</f>
-        <v>53.9</v>
+        <v>53.555</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4661,7 +4664,7 @@
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">C10/Assumptions!B5-1</f>
-        <v>0.195205175687314</v>
+        <v>0.185507141601639</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4728,15 +4731,15 @@
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">Summary!B6</f>
-        <v>22.3</v>
+        <v>21.9</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">Summary!C6</f>
-        <v>41.2094191925945</v>
+        <v>40.6746011363992</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">Summary!D6</f>
-        <v>66</v>
+        <v>65.4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4745,15 +4748,15 @@
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">Summary!B7</f>
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">Summary!C7</f>
-        <v>45.7882435473273</v>
+        <v>45.1940012626658</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">Summary!D7</f>
-        <v>68.8</v>
+        <v>68.1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4796,15 +4799,15 @@
       </c>
       <c r="B10" s="16" t="n">
         <f aca="false">Summary!B10</f>
-        <v>24.085</v>
+        <v>23.85</v>
       </c>
       <c r="C10" s="16" t="n">
         <f aca="false">Summary!C10</f>
-        <v>37.3501617402286</v>
+        <v>37.0470981750512</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">Summary!D10</f>
-        <v>53.9</v>
+        <v>53.555</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5023,7 +5026,7 @@
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B79+B80</f>
-        <v>28705.7</v>
+        <v>28060.65</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>61</v>
@@ -5825,7 +5828,7 @@
         <v>122</v>
       </c>
       <c r="B77" s="18" t="n">
-        <v>0.4258</v>
+        <v>0.4161</v>
       </c>
       <c r="C77" s="15" t="s">
         <v>123</v>
@@ -5845,7 +5848,7 @@
       </c>
       <c r="B79" s="8" t="n">
         <f aca="false">B76*B77*B78</f>
-        <v>28315.7</v>
+        <v>27670.65</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5941,7 +5944,7 @@
       </c>
       <c r="C8" s="23" t="n">
         <f aca="false">Assumptions!B79*Assumptions!B24</f>
-        <v>28315.7</v>
+        <v>27670.65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5963,7 +5966,7 @@
       <c r="B10" s="6"/>
       <c r="C10" s="22" t="n">
         <f aca="false">SUM(C6:C9)</f>
-        <v>49703.1383706237</v>
+        <v>49058.0883706237</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5973,7 +5976,7 @@
       <c r="B11" s="6"/>
       <c r="C11" s="10" t="n">
         <f aca="false">C10/Assumptions!B6</f>
-        <v>45.7882435473273</v>
+        <v>45.1940012626658</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5985,7 +5988,7 @@
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">-C10*Assumptions!B25</f>
-        <v>-4970.31383706237</v>
+        <v>-4905.80883706237</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5995,7 +5998,7 @@
       <c r="B13" s="6"/>
       <c r="C13" s="22" t="n">
         <f aca="false">C10+C12</f>
-        <v>44732.8245335614</v>
+        <v>44152.2795335614</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6005,7 +6008,7 @@
       <c r="B14" s="6"/>
       <c r="C14" s="16" t="n">
         <f aca="false">C13/Assumptions!B6</f>
-        <v>41.2094191925945</v>
+        <v>40.6746011363992</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6015,7 +6018,7 @@
       <c r="B15" s="6"/>
       <c r="C15" s="11" t="n">
         <f aca="false">C14/Assumptions!B5-1</f>
-        <v>0.318701414163025</v>
+        <v>0.301587236364775</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6027,7 +6030,7 @@
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">C8/C10</f>
-        <v>0.569696420150715</v>
+        <v>0.564038488229585</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6037,7 +6040,7 @@
       <c r="B17" s="6"/>
       <c r="C17" s="16" t="n">
         <f aca="false">C8*(1-Assumptions!B25)/Assumptions!B6</f>
-        <v>23.4768585905113</v>
+        <v>22.942040534316</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6045,12 +6048,12 @@
         <v>150</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="25" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="26" t="s">
         <v>152</v>
       </c>
@@ -6061,99 +6064,115 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="B22" s="28" t="n">
+      <c r="B22" s="8" t="n">
         <f aca="false">A22*Assumptions!$B$76*Assumptions!$B$78</f>
         <v>13300</v>
       </c>
-      <c r="C22" s="29" t="n">
+      <c r="C22" s="27" t="n">
         <f aca="false">((DCF!$B$25)+B22+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
         <v>28.7597370184812</v>
       </c>
-      <c r="D22" s="30" t="s">
+      <c r="D22" s="15" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="B23" s="28" t="n">
+      <c r="B23" s="8" t="n">
         <f aca="false">A23*Assumptions!$B$76*Assumptions!$B$78</f>
         <v>16625</v>
       </c>
-      <c r="C23" s="29" t="n">
+      <c r="C23" s="27" t="n">
         <f aca="false">((DCF!$B$25)+B23+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
         <v>31.5165311225807</v>
       </c>
-      <c r="D23" s="30"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="n">
+      <c r="D23" s="15"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="B24" s="28" t="n">
+      <c r="B24" s="8" t="n">
         <f aca="false">A24*Assumptions!$B$76*Assumptions!$B$78</f>
         <v>19950</v>
       </c>
-      <c r="C24" s="29" t="n">
+      <c r="C24" s="27" t="n">
         <f aca="false">((DCF!$B$25)+B24+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
         <v>34.2733252266802</v>
       </c>
-      <c r="D24" s="30"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="n">
+      <c r="D24" s="15"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="n">
         <v>0.3545</v>
       </c>
-      <c r="B25" s="28" t="n">
+      <c r="B25" s="8" t="n">
         <f aca="false">A25*Assumptions!$B$76*Assumptions!$B$78</f>
         <v>23574.25</v>
       </c>
-      <c r="C25" s="29" t="n">
+      <c r="C25" s="27" t="n">
         <f aca="false">((DCF!$B$25)+B25+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
         <v>37.2782308001486</v>
       </c>
-      <c r="D25" s="30" t="s">
+      <c r="D25" s="15" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="27" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="n">
         <v>0.4</v>
       </c>
-      <c r="B26" s="28" t="n">
+      <c r="B26" s="8" t="n">
         <f aca="false">A26*Assumptions!$B$76*Assumptions!$B$78</f>
         <v>26600</v>
       </c>
-      <c r="C26" s="29" t="n">
+      <c r="C26" s="27" t="n">
         <f aca="false">((DCF!$B$25)+B26+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
         <v>39.7869134348792</v>
       </c>
-      <c r="D26" s="30"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="n">
+      <c r="D26" s="15"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="n">
         <v>0.4258</v>
       </c>
-      <c r="B27" s="28" t="n">
+      <c r="B27" s="8" t="n">
         <f aca="false">A27*Assumptions!$B$76*Assumptions!$B$78</f>
         <v>28315.7</v>
       </c>
-      <c r="C27" s="29" t="n">
+      <c r="C27" s="27" t="n">
         <f aca="false">((DCF!$B$25)+B27+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
         <v>41.2094191925945</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="D27" s="15" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="30" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28" t="n">
+        <v>0.4161</v>
+      </c>
+      <c r="B28" s="29" t="n">
+        <f aca="false">A28*Assumptions!$B$76*Assumptions!$B$78</f>
+        <v>27670.65</v>
+      </c>
+      <c r="C28" s="30" t="n">
+        <f aca="false">((DCF!$B$25)+B28+Assumptions!$B$80+Assumptions!$B$21*Assumptions!$B$22)*(1-Assumptions!$B$25)/Assumptions!$B$6</f>
+        <v>40.6746011363992</v>
+      </c>
+      <c r="D28" s="31" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -6181,7 +6200,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6195,19 +6214,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -6226,8 +6245,8 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>164</v>
+      <c r="A6" s="32" t="s">
+        <v>165</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>26994</v>
@@ -6260,8 +6279,8 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
-        <v>164</v>
+      <c r="A7" s="32" t="s">
+        <v>165</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>26994</v>
@@ -6294,8 +6313,8 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
-        <v>165</v>
+      <c r="A8" s="32" t="s">
+        <v>166</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>16544.3</v>
@@ -6328,45 +6347,45 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="B9" s="32" t="n">
+      <c r="A9" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="B9" s="27" t="n">
         <f aca="false">B8/B7</f>
         <v>0.612888049196118</v>
       </c>
-      <c r="C9" s="32" t="n">
+      <c r="C9" s="27" t="n">
         <f aca="false">C8/C7</f>
         <v>0.86895321456604</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D9" s="27" t="n">
         <f aca="false">D8/D7</f>
         <v>0.934202801160077</v>
       </c>
-      <c r="E9" s="32" t="n">
+      <c r="E9" s="27" t="n">
         <f aca="false">D9*(1+Assumptions!$C$44)</f>
         <v>0.990254969229681</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="27" t="n">
         <f aca="false">E9*(1+Assumptions!$D$44)</f>
         <v>1.05957281707576</v>
       </c>
-      <c r="G9" s="32" t="n">
+      <c r="G9" s="27" t="n">
         <f aca="false">F9*(1+Assumptions!$E$44)</f>
         <v>1.13374291427106</v>
       </c>
-      <c r="H9" s="32" t="n">
+      <c r="H9" s="27" t="n">
         <f aca="false">G9*(1+Assumptions!$F$44)</f>
         <v>1.20176748912733</v>
       </c>
-      <c r="I9" s="32" t="n">
+      <c r="I9" s="27" t="n">
         <f aca="false">H9*(1+Assumptions!$G$44)</f>
         <v>1.27387353847497</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>167</v>
+      <c r="A10" s="32" t="s">
+        <v>168</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>2273</v>
@@ -6399,8 +6418,8 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
-        <v>168</v>
+      <c r="A11" s="32" t="s">
+        <v>169</v>
       </c>
       <c r="B11" s="17" t="n">
         <v>2323</v>
@@ -6433,8 +6452,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
-        <v>169</v>
+      <c r="A12" s="32" t="s">
+        <v>170</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>13610</v>
@@ -6467,8 +6486,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>170</v>
+      <c r="A13" s="32" t="s">
+        <v>171</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>854.2</v>
@@ -6501,8 +6520,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>171</v>
+      <c r="A14" s="32" t="s">
+        <v>172</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>2506.8</v>
@@ -6535,8 +6554,8 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>172</v>
+      <c r="A15" s="32" t="s">
+        <v>173</v>
       </c>
       <c r="B15" s="17" t="n">
         <v>7625.2</v>
@@ -6569,8 +6588,8 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>173</v>
+      <c r="A16" s="32" t="s">
+        <v>174</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>23854</v>
@@ -6603,8 +6622,8 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
-        <v>174</v>
+      <c r="A17" s="32" t="s">
+        <v>175</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>4950.9</v>
@@ -6637,8 +6656,8 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
-        <v>175</v>
+      <c r="A18" s="32" t="s">
+        <v>176</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>-487.7</v>
@@ -6671,8 +6690,8 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
-        <v>176</v>
+      <c r="A19" s="32" t="s">
+        <v>177</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">B16+B17+B18</f>
@@ -6708,8 +6727,8 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="31" t="s">
-        <v>177</v>
+      <c r="A21" s="32" t="s">
+        <v>178</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>5813.1</v>
@@ -6742,7 +6761,7 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="32" t="s">
         <v>98</v>
       </c>
       <c r="B22" s="14" t="n">
@@ -6779,8 +6798,8 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
-        <v>178</v>
+      <c r="A23" s="32" t="s">
+        <v>179</v>
       </c>
       <c r="B23" s="17" t="n">
         <v>3460.9</v>
@@ -6813,8 +6832,8 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31" t="s">
-        <v>179</v>
+      <c r="A24" s="32" t="s">
+        <v>180</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>374.3</v>
@@ -6847,8 +6866,8 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
-        <v>180</v>
+      <c r="A25" s="32" t="s">
+        <v>181</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>3794.6</v>
@@ -6881,8 +6900,8 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
-        <v>181</v>
+      <c r="A26" s="32" t="s">
+        <v>182</v>
       </c>
       <c r="B26" s="14" t="n">
         <f aca="false">B25/B16</f>
@@ -6918,8 +6937,8 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="31" t="s">
-        <v>182</v>
+      <c r="A27" s="32" t="s">
+        <v>183</v>
       </c>
       <c r="B27" s="17" t="n">
         <v>243.7</v>
@@ -6932,8 +6951,8 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="31" t="s">
-        <v>183</v>
+      <c r="A28" s="32" t="s">
+        <v>184</v>
       </c>
       <c r="B28" s="17" t="n">
         <v>1207.6</v>
@@ -6946,8 +6965,8 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="31" t="s">
-        <v>184</v>
+      <c r="A29" s="32" t="s">
+        <v>185</v>
       </c>
       <c r="B29" s="17" t="n">
         <v>8980.5</v>
@@ -6961,7 +6980,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -6990,7 +7009,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7001,7 +7020,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7009,18 +7028,18 @@
         <v>33</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">Assumptions!B27*Assumptions!B28/Assumptions!B6</f>
@@ -7029,7 +7048,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">Assumptions!B27/Assumptions!B6</f>
@@ -7038,7 +7057,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">'Income Statement'!E26/Assumptions!B6</f>
@@ -7047,10 +7066,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">Assumptions!B29*Assumptions!B30/Assumptions!B6</f>
@@ -7059,7 +7078,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">Assumptions!B29/Assumptions!B6</f>
@@ -7068,7 +7087,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">Assumptions!B5/('Balance Sheet'!D16/Assumptions!B6)</f>
@@ -7100,7 +7119,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7112,7 +7131,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7134,7 +7153,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B6" s="23" t="n">
         <f aca="false">Segments!E16</f>
@@ -7159,7 +7178,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B7" s="23" t="n">
         <f aca="false">Segments!E25</f>
@@ -7184,7 +7203,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B8" s="23" t="n">
         <f aca="false">-Segments!E24</f>
@@ -7209,7 +7228,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B9" s="23" t="n">
         <f aca="false">Segments!E23</f>
@@ -7234,7 +7253,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B9*(1-Assumptions!$B$7)</f>
@@ -7259,7 +7278,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B11" s="23" t="n">
         <f aca="false">Segments!E24</f>
@@ -7284,7 +7303,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">-Assumptions!$C$57</f>
@@ -7309,7 +7328,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B13" s="23" t="n">
         <f aca="false">-'Balance Sheet'!E31</f>
@@ -7334,7 +7353,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">SUM(B10:B13)</f>
@@ -7359,7 +7378,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B15" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$16)^1</f>
@@ -7384,7 +7403,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">B14*B15</f>
@@ -7409,7 +7428,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">SUM(B16:F16)</f>
@@ -7418,7 +7437,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">F14*(1+Assumptions!$B$17)/(Assumptions!$B$16-Assumptions!$B$17)</f>
@@ -7427,7 +7446,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B19*F15</f>
@@ -7436,7 +7455,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">B18+B20</f>
@@ -7445,7 +7464,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B22" s="24" t="n">
         <f aca="false">B20/B21</f>
@@ -7454,7 +7473,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">-Assumptions!$B$19</f>
@@ -7463,7 +7482,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">-Assumptions!$B$20</f>
@@ -7472,7 +7491,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B25" s="22" t="n">
         <f aca="false">B21-Assumptions!$B$19-Assumptions!$B$20</f>
@@ -7481,7 +7500,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">0.01*(1-Assumptions!$B$7)*(SUMPRODUCT(B6:F6,B15:F15)+F6*(1+Assumptions!$B$17)/(Assumptions!$B$16-Assumptions!$B$17)*F15)</f>
@@ -7490,7 +7509,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -7518,7 +7537,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -7532,19 +7551,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>84</v>
@@ -7564,7 +7583,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>23854</v>
@@ -7598,7 +7617,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B7" s="17" t="n">
         <v>4950.9</v>
@@ -7632,7 +7651,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>-487.7</v>
@@ -7666,7 +7685,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B9" s="35" t="n">
         <v>28317.2</v>
@@ -7700,7 +7719,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>6884.3</v>
@@ -7734,7 +7753,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">B10/B9</f>
@@ -7771,7 +7790,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>-3430.8</v>
@@ -7805,7 +7824,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>518.8</v>
@@ -7839,7 +7858,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>-268.9</v>
@@ -7873,7 +7892,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B15" s="35" t="n">
         <v>3703.4</v>
@@ -7907,7 +7926,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>1066.1</v>
@@ -7941,7 +7960,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B17" s="35" t="n">
         <v>4769.5</v>
@@ -7975,7 +7994,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>820</v>
@@ -8009,7 +8028,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">B17+B18</f>
@@ -8046,7 +8065,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>-1499.2</v>
@@ -8080,7 +8099,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>-965.8</v>
@@ -8114,7 +8133,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B22" s="35" t="n">
         <v>2304.4</v>
@@ -8148,7 +8167,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B23" s="17" t="n">
         <v>-493.2</v>
@@ -8182,7 +8201,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B24" s="35" t="n">
         <v>1811.2</v>
@@ -8216,7 +8235,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B25" s="17" t="n">
         <v>79.5</v>
@@ -8250,7 +8269,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B26" s="35" t="n">
         <v>1890.8</v>
@@ -8284,7 +8303,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B27" s="14" t="n">
         <f aca="false">B26/B9</f>
@@ -8321,7 +8340,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>